<commit_message>
Atualiza documentacao e artefatos do FACIN_IA
</commit_message>
<xml_diff>
--- a/docs/FACIN_IA_Avaliacao_Automatica.xlsx
+++ b/docs/FACIN_IA_Avaliacao_Automatica.xlsx
@@ -467,7 +467,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. O score da dimensão é ponderado pelos pesos internos dos indicadores.</t>
+          <t>3. A pontuação da dimensão é ponderada pelos pesos internos dos indicadores.</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -682,7 +682,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
@@ -727,7 +727,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -772,7 +772,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
@@ -817,7 +817,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -862,7 +862,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
@@ -907,7 +907,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
@@ -952,7 +952,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -997,7 +997,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cobertura de testes e validações de IA no pipeline</t>
+          <t>Cobertura de testes e validações de IA na esteira</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>menor_melhor</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
@@ -1532,7 +1532,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cobertura de testes e validações de IA no pipeline</t>
+          <t>Cobertura de testes e validações de IA na esteira</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>menor_melhor</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>maior_melhor</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Score_dimensão</t>
+          <t>Pontuação_dimensão</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Menor score geral</t>
+          <t>Menor pontuação geral</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>

</xml_diff>